<commit_message>
Corrige sigla 26620: DMAFE para DEMAFE
</commit_message>
<xml_diff>
--- a/CODIGOS_CENTRO_DE_CUSTO_SISERGE_2025_CORRIGIDA.xlsx
+++ b/CODIGOS_CENTRO_DE_CUSTO_SISERGE_2025_CORRIGIDA.xlsx
@@ -614,12 +614,12 @@
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1" s="4">
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="0" t="inlineStr">
         <is>
           <t>PREDIO CENTRAL - SALA DE TELECOM</t>
         </is>
       </c>
-      <c r="E26" t="n">
+      <c r="E26" s="0" t="n">
         <v>20023</v>
       </c>
     </row>
@@ -1089,19 +1089,19 @@
       </c>
     </row>
     <row r="75" ht="15.75" customHeight="1" s="4">
-      <c r="A75" t="inlineStr">
+      <c r="A75" s="0" t="inlineStr">
         <is>
           <t>DEPARTAMENTOS</t>
         </is>
       </c>
     </row>
     <row r="76" ht="15.75" customHeight="1" s="4">
-      <c r="B76" t="inlineStr">
+      <c r="B76" s="0" t="inlineStr">
         <is>
           <t>DEPARTAMENTOS</t>
         </is>
       </c>
-      <c r="E76" t="n">
+      <c r="E76" s="0" t="n">
         <v>26000</v>
       </c>
     </row>
@@ -2409,7 +2409,7 @@
     <row r="211" ht="15.75" customHeight="1" s="4">
       <c r="B211" s="3" t="inlineStr">
         <is>
-          <t>DMAFE - IPCA - LAB PESQUISA ENS DE MAT - LAPEM</t>
+          <t>DEMAFE - IPCA - LAB PESQUISA ENS DE MAT - LAPEM</t>
         </is>
       </c>
       <c r="E211" s="3" t="n">
@@ -2581,12 +2581,12 @@
       </c>
     </row>
     <row r="229" ht="15.75" customHeight="1" s="4">
-      <c r="C229" t="inlineStr">
+      <c r="C229" s="0" t="inlineStr">
         <is>
           <t>DZO - PREDIO DA ZOOTECNIA - VARANDA E CORREDORES</t>
         </is>
       </c>
-      <c r="E229" t="n">
+      <c r="E229" s="0" t="n">
         <v>26716</v>
       </c>
     </row>
@@ -2811,82 +2811,82 @@
       </c>
     </row>
     <row r="252" ht="15.75" customHeight="1" s="4">
-      <c r="B252" t="inlineStr">
+      <c r="B252" s="0" t="inlineStr">
         <is>
           <t>DZO - GALPAO EXPERIMENTAL DE BOVINOCULTURA</t>
         </is>
       </c>
-      <c r="E252" t="n">
+      <c r="E252" s="0" t="n">
         <v>26738</v>
       </c>
     </row>
     <row r="253" ht="15.75" customHeight="1" s="4">
-      <c r="B253" t="inlineStr">
+      <c r="B253" s="0" t="inlineStr">
         <is>
           <t>DZO - CUNICULTURA - COELHOS</t>
         </is>
       </c>
-      <c r="E253" t="n">
+      <c r="E253" s="0" t="n">
         <v>26739</v>
       </c>
     </row>
     <row r="254" ht="15.75" customHeight="1" s="4">
-      <c r="B254" t="inlineStr">
+      <c r="B254" s="0" t="inlineStr">
         <is>
           <t>DZO - LABORATORIO OVINOCAPRINOCULTURA</t>
         </is>
       </c>
-      <c r="E254" t="n">
+      <c r="E254" s="0" t="n">
         <v>26740</v>
       </c>
     </row>
     <row r="255" ht="15.75" customHeight="1" s="4">
-      <c r="B255" t="inlineStr">
+      <c r="B255" s="0" t="inlineStr">
         <is>
           <t>DZO - FRANGO - CORTE</t>
         </is>
       </c>
-      <c r="E255" t="n">
+      <c r="E255" s="0" t="n">
         <v>26741</v>
       </c>
     </row>
     <row r="256" ht="15.75" customHeight="1" s="4">
-      <c r="B256" t="inlineStr">
+      <c r="B256" s="0" t="inlineStr">
         <is>
           <t>DZO - CAPRINOCULTURA</t>
         </is>
       </c>
-      <c r="E256" t="n">
+      <c r="E256" s="0" t="n">
         <v>26742</v>
       </c>
     </row>
     <row r="257" ht="15.75" customHeight="1" s="4">
-      <c r="B257" t="inlineStr">
+      <c r="B257" s="0" t="inlineStr">
         <is>
           <t>DZO - DEPOSITOS E SALA DE APOIO LAB OVINOCAPRINO</t>
         </is>
       </c>
-      <c r="E257" t="n">
+      <c r="E257" s="0" t="n">
         <v>26743</v>
       </c>
     </row>
     <row r="258" ht="15.75" customHeight="1" s="4">
-      <c r="B258" t="inlineStr">
+      <c r="B258" s="0" t="inlineStr">
         <is>
           <t>DZO - APICULTURA</t>
         </is>
       </c>
-      <c r="E258" t="n">
+      <c r="E258" s="0" t="n">
         <v>26744</v>
       </c>
     </row>
     <row r="259" ht="15.75" customHeight="1" s="4">
-      <c r="B259" t="inlineStr">
+      <c r="B259" s="0" t="inlineStr">
         <is>
           <t>DZO - SEMOVENTES</t>
         </is>
       </c>
-      <c r="E259" t="n">
+      <c r="E259" s="0" t="n">
         <v>26745</v>
       </c>
     </row>
@@ -3223,12 +3223,12 @@
       </c>
     </row>
     <row r="295" ht="15.75" customHeight="1" s="4">
-      <c r="B295" t="inlineStr">
+      <c r="B295" s="0" t="inlineStr">
         <is>
           <t>COORDENACAO GERAL DE ADMINISTRACAO E FINANCAS</t>
         </is>
       </c>
-      <c r="E295" t="n">
+      <c r="E295" s="0" t="n">
         <v>31000</v>
       </c>
     </row>
@@ -3387,22 +3387,22 @@
       </c>
     </row>
     <row r="312" ht="15.75" customHeight="1" s="4">
-      <c r="C312" t="inlineStr">
+      <c r="C312" s="0" t="inlineStr">
         <is>
           <t>PATRIMONIO - GALPAO 3 - IRRECUPERAVEL/ANTIECONOMIC</t>
         </is>
       </c>
-      <c r="E312" t="n">
+      <c r="E312" s="0" t="n">
         <v>31212</v>
       </c>
     </row>
     <row r="313" ht="15.75" customHeight="1" s="4">
-      <c r="C313" t="inlineStr">
+      <c r="C313" s="0" t="inlineStr">
         <is>
           <t>PATRIMONIO - GALPAO 3</t>
         </is>
       </c>
-      <c r="E313" t="n">
+      <c r="E313" s="0" t="n">
         <v>31213</v>
       </c>
     </row>
@@ -4462,22 +4462,22 @@
       </c>
     </row>
     <row r="424" ht="15.75" customHeight="1" s="4">
-      <c r="B424" t="inlineStr">
+      <c r="B424" s="0" t="inlineStr">
         <is>
           <t>SALA WEB RADIO (ALOJAMENTO / BLOCO B / SALA 1)</t>
         </is>
       </c>
-      <c r="E424" t="n">
+      <c r="E424" s="0" t="n">
         <v>70040</v>
       </c>
     </row>
     <row r="425" ht="15.75" customHeight="1" s="4">
-      <c r="B425" t="inlineStr">
+      <c r="B425" s="0" t="inlineStr">
         <is>
           <t>CAPELA / IGREJINHA</t>
         </is>
       </c>
-      <c r="E425" t="n">
+      <c r="E425" s="0" t="n">
         <v>70041</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Alinha descricoes ao ODS: sigla DMAFE, EFI, DZO salas 7-9
</commit_message>
<xml_diff>
--- a/CODIGOS_CENTRO_DE_CUSTO_SISERGE_2025_CORRIGIDA.xlsx
+++ b/CODIGOS_CENTRO_DE_CUSTO_SISERGE_2025_CORRIGIDA.xlsx
@@ -2209,7 +2209,7 @@
     <row r="191" ht="15.75" customHeight="1" s="4">
       <c r="B191" s="3" t="inlineStr">
         <is>
-          <t>DEMAFE - DEP. ACADEMICO DE MATEMATICA E FISICA</t>
+          <t>DMAFE - DEP. ACADEMICO DE MATEMATICA E FISICA</t>
         </is>
       </c>
       <c r="E191" s="3" t="n">
@@ -2219,7 +2219,7 @@
     <row r="192" ht="15.75" customHeight="1" s="4">
       <c r="B192" s="3" t="inlineStr">
         <is>
-          <t>DEMAFE - LABORATORIO DE FISICA</t>
+          <t>DMAFE - LABORATORIO DE FISICA</t>
         </is>
       </c>
       <c r="E192" s="3" t="n">
@@ -2229,7 +2229,7 @@
     <row r="193" ht="15.75" customHeight="1" s="4">
       <c r="B193" s="3" t="inlineStr">
         <is>
-          <t>DEMAFE - LABORATORIO DE INFORMÁTICA</t>
+          <t>DMAFE - LABORATORIO DE INFORMÁTICA</t>
         </is>
       </c>
       <c r="E193" s="3" t="n">
@@ -2239,7 +2239,7 @@
     <row r="194" ht="15.75" customHeight="1" s="4">
       <c r="B194" s="3" t="inlineStr">
         <is>
-          <t>DEMAFE - LABORATÓRIO DE MATEMÁTICA</t>
+          <t>DMAFE - LABORATÓRIO DE MATEMÁTICA</t>
         </is>
       </c>
       <c r="E194" s="3" t="n">
@@ -2249,7 +2249,7 @@
     <row r="195" ht="15.75" customHeight="1" s="4">
       <c r="B195" s="3" t="inlineStr">
         <is>
-          <t>DEMAFE - SALA DOS PROFESSORES 2</t>
+          <t>DMAFE - SALA DOS PROFESSORES 2</t>
         </is>
       </c>
       <c r="E195" s="3" t="n">
@@ -2259,7 +2259,7 @@
     <row r="196" ht="15.75" customHeight="1" s="4">
       <c r="B196" s="3" t="inlineStr">
         <is>
-          <t>DEMAFE - SALA DOS PROFESSORES 2 - GABINETE 1</t>
+          <t>DMAFE - SALA DOS PROFESSORES 2 - GABINETE 1</t>
         </is>
       </c>
       <c r="E196" s="3" t="n">
@@ -2269,7 +2269,7 @@
     <row r="197" ht="15.75" customHeight="1" s="4">
       <c r="B197" s="3" t="inlineStr">
         <is>
-          <t>DEMAFE - SALA DOS PROFESSORES 2 - GABINETE 2</t>
+          <t>DMAFE - SALA DOS PROFESSORES 2 - GABINETE 2</t>
         </is>
       </c>
       <c r="E197" s="3" t="n">
@@ -2279,7 +2279,7 @@
     <row r="198" ht="15.75" customHeight="1" s="4">
       <c r="B198" s="3" t="inlineStr">
         <is>
-          <t>DEMAFE - SALA DOS PROFESSORES 2 - GABINETE 3</t>
+          <t>DMAFE - SALA DOS PROFESSORES 2 - GABINETE 3</t>
         </is>
       </c>
       <c r="E198" s="3" t="n">
@@ -2289,7 +2289,7 @@
     <row r="199" ht="15.75" customHeight="1" s="4">
       <c r="B199" s="3" t="inlineStr">
         <is>
-          <t>DEMAFE - SALA DOS PROFESSORES 2 - GABINETE 4</t>
+          <t>DMAFE - SALA DOS PROFESSORES 2 - GABINETE 4</t>
         </is>
       </c>
       <c r="E199" s="3" t="n">
@@ -2299,7 +2299,7 @@
     <row r="200" ht="15.75" customHeight="1" s="4">
       <c r="B200" s="3" t="inlineStr">
         <is>
-          <t>DEMAFE - SALA DOS PROFESSORES 2 - GABINETE REUNIÃO</t>
+          <t>DMAFE - SALA DOS PROFESSORES 2 - GABINETE REUNIÃO</t>
         </is>
       </c>
       <c r="E200" s="3" t="n">
@@ -2309,7 +2309,7 @@
     <row r="201" ht="15.75" customHeight="1" s="4">
       <c r="B201" s="3" t="inlineStr">
         <is>
-          <t>DEMAFE - SALA DOS PROFESSORES 3</t>
+          <t>DMAFE - SALA DOS PROFESSORES 3</t>
         </is>
       </c>
       <c r="E201" s="3" t="n">
@@ -2319,7 +2319,7 @@
     <row r="202" ht="15.75" customHeight="1" s="4">
       <c r="B202" s="3" t="inlineStr">
         <is>
-          <t>DEMAFE - SALA DOS PROFESSORES 3 - GABINETE 1</t>
+          <t>DMAFE - SALA DOS PROFESSORES 3 - GABINETE 1</t>
         </is>
       </c>
       <c r="E202" s="3" t="n">
@@ -2329,7 +2329,7 @@
     <row r="203" ht="15.75" customHeight="1" s="4">
       <c r="B203" s="3" t="inlineStr">
         <is>
-          <t>DEMAFE - SALA DOS PROFESSORES 3 - GABINETE 2</t>
+          <t>DMAFE - SALA DOS PROFESSORES 3 - GABINETE 2</t>
         </is>
       </c>
       <c r="E203" s="3" t="n">
@@ -2339,7 +2339,7 @@
     <row r="204" ht="15.75" customHeight="1" s="4">
       <c r="B204" s="3" t="inlineStr">
         <is>
-          <t>DEMAFE - SALA DOS PROFESSORES 3 - GABINETE 3</t>
+          <t>DMAFE - SALA DOS PROFESSORES 3 - GABINETE 3</t>
         </is>
       </c>
       <c r="E204" s="3" t="n">
@@ -2349,7 +2349,7 @@
     <row r="205" ht="15.75" customHeight="1" s="4">
       <c r="B205" s="3" t="inlineStr">
         <is>
-          <t>DEMAFE - SALA DOS PROFESSORES 3 - GABINETE 4</t>
+          <t>DMAFE - SALA DOS PROFESSORES 3 - GABINETE 4</t>
         </is>
       </c>
       <c r="E205" s="3" t="n">
@@ -2359,7 +2359,7 @@
     <row r="206" ht="15.75" customHeight="1" s="4">
       <c r="B206" s="3" t="inlineStr">
         <is>
-          <t>DEMAFE - SALA DOS PROFESSORES 3 - GABINETE 5</t>
+          <t>DMAFE - SALA DOS PROFESSORES 3 - GABINETE 5</t>
         </is>
       </c>
       <c r="E206" s="3" t="n">
@@ -2369,7 +2369,7 @@
     <row r="207" ht="15.75" customHeight="1" s="4">
       <c r="B207" s="3" t="inlineStr">
         <is>
-          <t>DEMAFE - SALA DOS PROFESSORES 3 - GABINETE 6</t>
+          <t>DMAFE - SALA DOS PROFESSORES 3 - GABINETE 6</t>
         </is>
       </c>
       <c r="E207" s="3" t="n">
@@ -2409,7 +2409,7 @@
     <row r="211" ht="15.75" customHeight="1" s="4">
       <c r="B211" s="3" t="inlineStr">
         <is>
-          <t>DEMAFE - IPCA - LAB PESQUISA ENS DE MAT - LAPEM</t>
+          <t>DMAFE - IPCA - LAB PESQUISA ENS DE MAT - LAPEM</t>
         </is>
       </c>
       <c r="E211" s="3" t="n">
@@ -2486,7 +2486,7 @@
     <row r="219" ht="15.75" customHeight="1" s="4">
       <c r="B219" s="3" t="inlineStr">
         <is>
-          <t>DZO - SALA DE PROFESSORES E REUNIÃO</t>
+          <t>DZO - SALA 7</t>
         </is>
       </c>
       <c r="E219" s="3" t="n">
@@ -2496,7 +2496,7 @@
     <row r="220" ht="15.75" customHeight="1" s="4">
       <c r="B220" s="3" t="inlineStr">
         <is>
-          <t>DZO - SALA 6</t>
+          <t>DZO - SALA 8</t>
         </is>
       </c>
       <c r="E220" s="3" t="n">
@@ -2506,7 +2506,7 @@
     <row r="221" ht="15.75" customHeight="1" s="4">
       <c r="B221" s="3" t="inlineStr">
         <is>
-          <t>DZO - SALA 7</t>
+          <t>DZO - SALA 9</t>
         </is>
       </c>
       <c r="E221" s="3" t="n">
@@ -2900,7 +2900,7 @@
     <row r="261" ht="15.75" customHeight="1" s="4">
       <c r="B261" s="3" t="inlineStr">
         <is>
-          <t>NEFI - NUCLEO DE EDUCACAO FISICA</t>
+          <t>EFI - NUCLEO DE EDUCACAO FISICA</t>
         </is>
       </c>
       <c r="E261" s="3" t="n">

</xml_diff>

<commit_message>
Alinha ao ODS: 23000, 26110, 26717, 31205
</commit_message>
<xml_diff>
--- a/CODIGOS_CENTRO_DE_CUSTO_SISERGE_2025_CORRIGIDA.xlsx
+++ b/CODIGOS_CENTRO_DE_CUSTO_SISERGE_2025_CORRIGIDA.xlsx
@@ -656,14 +656,14 @@
     <row r="30" ht="15.75" customHeight="1" s="4">
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>COORDENACAO GERAL DE ASSUNTOS E REGISTROS ACADEMIC</t>
+          <t>COORD. GERAL DE REGISTROS ACADÊMICOS</t>
         </is>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1" s="4">
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>COORDENACAO GERAL DE ASSUNTOS E REGISTROS ACADEMIC</t>
+          <t>COORD. GERAL DE REGISTROS ACADÊMICOS</t>
         </is>
       </c>
       <c r="E31" s="3" t="n">
@@ -1252,7 +1252,7 @@
     <row r="92" ht="15.75" customHeight="1" s="4">
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>DAAA - AGRICULTURA - SALA PROFESSORES (AO LADO DA SALA 4)</t>
+          <t>DAAA - AGRICULTURA - SALA PROFESSOR (SALA4)</t>
         </is>
       </c>
       <c r="E92" s="3" t="n">
@@ -2593,7 +2593,7 @@
     <row r="230" ht="15.75" customHeight="1" s="4">
       <c r="C230" s="3" t="inlineStr">
         <is>
-          <t>DZO - PREDIO DA ZOOTECNIA - SALA 9</t>
+          <t>DZO - PREDIO DA ZOOTECNIA - COZ / SALA / DEPOSITO</t>
         </is>
       </c>
       <c r="E230" s="3" t="n">
@@ -3319,7 +3319,7 @@
     <row r="305" ht="15.75" customHeight="1" s="4">
       <c r="C305" s="3" t="inlineStr">
         <is>
-          <t>PATRIMONIO - GALPAO 2 - IRRECUPERÁVEL</t>
+          <t>GALPAO 2 - IRRECUPERAVEL/ANTIECONOMICO</t>
         </is>
       </c>
       <c r="E305" s="3" t="n">

</xml_diff>